<commit_message>
updated the name and conftest
</commit_message>
<xml_diff>
--- a/test_data/AWX_Bank_Transfer_testing_v3_Latest.xlsx
+++ b/test_data/AWX_Bank_Transfer_testing_v3_Latest.xlsx
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="I4" s="103" t="n">
-        <v>311</v>
+        <v>411</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2612145</v>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="Y4" s="22" t="n"/>
       <c r="Z4" s="103" t="n">
-        <v>311</v>
+        <v>411</v>
       </c>
       <c r="AA4" s="22" t="n"/>
       <c r="AB4" s="22" t="n"/>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="I5" s="103" t="n">
-        <v>322</v>
+        <v>422</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2612145</v>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="Y5" s="22" t="n"/>
       <c r="Z5" s="103" t="n">
-        <v>322</v>
+        <v>422</v>
       </c>
       <c r="AA5" s="22" t="n"/>
       <c r="AB5" s="22" t="n"/>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="I6" s="103" t="n">
-        <v>333</v>
+        <v>433</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2612145</v>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="Y6" s="22" t="n"/>
       <c r="Z6" s="103" t="n">
-        <v>333</v>
+        <v>433</v>
       </c>
       <c r="AA6" s="22" t="n"/>
       <c r="AB6" s="22" t="n"/>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="I7" s="103" t="n">
-        <v>344</v>
+        <v>444</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2612145</v>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="Y7" s="22" t="n"/>
       <c r="Z7" s="103" t="n">
-        <v>344</v>
+        <v>444</v>
       </c>
       <c r="AA7" s="22" t="n"/>
       <c r="AB7" s="22" t="n"/>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="I8" s="103" t="n">
-        <v>355</v>
+        <v>455</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>2612145</v>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="Y8" s="22" t="n"/>
       <c r="Z8" s="103" t="n">
-        <v>355</v>
+        <v>455</v>
       </c>
       <c r="AA8" s="22" t="n"/>
       <c r="AB8" s="22" t="n"/>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="I9" s="103" t="n">
-        <v>366</v>
+        <v>466</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2612145</v>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="Y9" s="22" t="n"/>
       <c r="Z9" s="103" t="n">
-        <v>366</v>
+        <v>466</v>
       </c>
       <c r="AA9" s="22" t="n"/>
       <c r="AB9" s="22" t="n"/>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="I10" s="103" t="n">
-        <v>377</v>
+        <v>477</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2612145</v>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="Y10" s="22" t="n"/>
       <c r="Z10" s="103" t="n">
-        <v>377</v>
+        <v>477</v>
       </c>
       <c r="AA10" s="22" t="n"/>
       <c r="AB10" s="22" t="n"/>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="I11" s="103" t="n">
-        <v>388</v>
+        <v>488</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>2612145</v>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="Y11" s="22" t="n"/>
       <c r="Z11" s="103" t="n">
-        <v>388</v>
+        <v>488</v>
       </c>
       <c r="AA11" s="22" t="n"/>
       <c r="AB11" s="22" t="n"/>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="I12" s="103" t="n">
-        <v>399</v>
+        <v>499</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2612145</v>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="Y12" s="22" t="n"/>
       <c r="Z12" s="103" t="n">
-        <v>399</v>
+        <v>499</v>
       </c>
       <c r="AA12" s="22" t="n"/>
       <c r="AB12" s="22" t="inlineStr">
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="I13" s="103" t="n">
-        <v>410</v>
+        <v>510</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>2612145</v>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Y13" s="22" t="n"/>
       <c r="Z13" s="103" t="n">
-        <v>410</v>
+        <v>510</v>
       </c>
       <c r="AA13" s="22" t="n"/>
       <c r="AB13" s="22" t="n"/>

</xml_diff>